<commit_message>
Add QR code generation and phishing dataset updates
- Implemented QR code generation from CSV dataset in `generateQR.py`.
- Added new QR test cases images for URLs.
- Created a new CSV file `dataset(2).csv` with a phishing URL for testing.
- Updated the main `dataset.csv` with various safe and phishing URLs.
- Introduced `generate_industry_test_link.py` to append industry standard test links to the dataset.
- Developed `generate_phish_link.py` to fetch live phishing URLs and classify them based on attack vectors.
</commit_message>
<xml_diff>
--- a/googleLens_scanner_automation/QR_Scanner_Test_Log.xlsx
+++ b/googleLens_scanner_automation/QR_Scanner_Test_Log.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:L202"/>
+  <dimension ref="A2:L203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -10955,6 +10955,58 @@
       <c r="L202" s="6" t="inlineStr">
         <is>
           <t>Diblokir (Error UI: Timeout/Terhalang Pop-up)</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="6" t="n">
+        <v>201</v>
+      </c>
+      <c r="B203" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:54:49</t>
+        </is>
+      </c>
+      <c r="C203" s="7" t="inlineStr">
+        <is>
+          <t>https://composerprogrammer.com/introductiontocomputermusic.pdf</t>
+        </is>
+      </c>
+      <c r="D203" s="6" t="inlineStr">
+        <is>
+          <t>safe</t>
+        </is>
+      </c>
+      <c r="E203" s="6" t="inlineStr">
+        <is>
+          <t>Live Safe (Tech News)</t>
+        </is>
+      </c>
+      <c r="F203" s="6" t="inlineStr">
+        <is>
+          <t>Aman</t>
+        </is>
+      </c>
+      <c r="G203" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H203" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I203" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J203" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K203" s="6" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="L203" s="6" t="inlineStr">
+        <is>
+          <t>Tembus total. Halaman termuat dengan sukses.</t>
         </is>
       </c>
     </row>

</xml_diff>